<commit_message>
version 5 further split power 22 V and 6 V 2-pcbs
</commit_message>
<xml_diff>
--- a/Laser_Driver_v4/Mains_18V_TEC/Mains_18V_TEC_BOM.xlsx
+++ b/Laser_Driver_v4/Mains_18V_TEC/Mains_18V_TEC_BOM.xlsx
@@ -1040,16 +1040,26 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>RC0805FR-0710RL</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>YAGEO</t>
+        </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>R32, R33</t>
+          <t>R40, R41, R42, R43</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>4.75R 2W | RESC3263X80N</t>
+          <t>10 ohm 1% 0805 | base-stopper (anti-parasitic), 1 per MJL pass transistor</t>
         </is>
       </c>
     </row>
@@ -1135,32 +1145,32 @@
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>HSE-B18254-0396H</t>
+          <t>657-10ABPE</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Same Sky (CUI Devices)</t>
+          <t>Wakefield Thermal Solutions</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Q7, Q8, Q9, Q10, D7</t>
+          <t>Q7, Q8, Q9, Q10</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Heatsink 42mm 2.29C/W@200LFM (forced air) | 1 per power device</t>
+          <t>Vertical board-mount heat sink TO-247/TO-264, 41.9x25.4mm base, 25.4mm tall, 3.7C/W @200LFM (6.8C/W nat), bolt-on w/ 2 wave-solder pins | 1 per device</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
@@ -1174,7 +1184,7 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Q7, Q8, Q9, Q10, D7</t>
+          <t>Q7, Q8, Q9, Q10</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">

</xml_diff>